<commit_message>
update code, release app
</commit_message>
<xml_diff>
--- a/data_template.xlsx
+++ b/data_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="3264" windowHeight="23260"/>
+    <workbookView windowHeight="15460"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
     <t>107096649442</t>
   </si>
   <si>
-    <t>03PL</t>
+    <t>HQHUNGYEN</t>
   </si>
   <si>
     <t>107096646160</t>

</xml_diff>